<commit_message>
Automation testing Day 4
</commit_message>
<xml_diff>
--- a/SprintWorkspace/NoBroker/target/classes/ExcelData/FormData.xlsx
+++ b/SprintWorkspace/NoBroker/target/classes/ExcelData/FormData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Windows\System32\config\systemprofile\SprintWorkspace\NoBroker\src\test\resource\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7ED4BA5-BC4B-40C7-86E2-3A5F7EE714EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D912EE-9B03-47A7-BC14-8B25C03DF0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Name</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>Pune</t>
+  </si>
+  <si>
+    <t>9865432190</t>
+  </si>
+  <si>
+    <t>50</t>
   </si>
 </sst>
 </file>
@@ -99,9 +105,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -420,14 +427,14 @@
       <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2">
-        <v>9865432190</v>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2">
-        <v>50</v>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>